<commit_message>
separamos streamlit y API
</commit_message>
<xml_diff>
--- a/Produccion Astroflores BL25-26-27-28 a la Semana 09.xlsx
+++ b/Produccion Astroflores BL25-26-27-28 a la Semana 09.xlsx
@@ -547,7 +547,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -561,9 +561,9 @@
   <cols>
     <col min="1" max="1" width="7.75" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="2" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="13.125" style="2" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.375" style="2" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.375" style="2" customWidth="1"/>
     <col min="6" max="7" width="14.625" style="2" customWidth="1"/>
     <col min="8" max="8" width="13" style="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14" style="2" customWidth="1"/>

</xml_diff>